<commit_message>
Populate repechage and final sheets in official export
</commit_message>
<xml_diff>
--- a/resources/tir_qualif_template.xlsx
+++ b/resources/tir_qualif_template.xlsx
@@ -7,11 +7,15 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TIR QUALIFICATION" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TIR REPECHAGE" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TIR FINAL " sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="FromArray_1">_xlfn.ANCHORARRAY('TIR QUALIFICATION'!$AJ$10)</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'TIR QUALIFICATION'!$2:$9</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'TIR QUALIFICATION'!$AJ$2:$BN$52</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'TIR REPECHAGE'!$A$1:$AM$41</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'TIR FINAL '!$B$1:$AC$19</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -6200,7 +6204,7 @@
     <xf numFmtId="0" fontId="55" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="73" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="686">
+  <cellXfs count="735">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center"/>
@@ -8778,6 +8782,117 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="8" borderId="386" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="294" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="295" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="8" borderId="351" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="305" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="306" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="307" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="387" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="310" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="8" borderId="388" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="315" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="317" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="318" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="35" fillId="8" borderId="389" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="9" borderId="385" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="375" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="6" borderId="385" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="385" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="321" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="322" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="383" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="324" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="325" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="326" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="382" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="right" vertical="center" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="324" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="right" vertical="center" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="344" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="right" vertical="center" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="329" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="329" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="333" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="359" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="360" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="306" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="334" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="394" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="74" fillId="3" borderId="372" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="379" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="380" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="10" borderId="392" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="3">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="351" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="74" fillId="10" borderId="372" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -9356,6 +9471,313 @@
     </pic>
     <clientData/>
   </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>9</col>
+      <colOff>123827</colOff>
+      <row>12</row>
+      <rowOff>47625</rowOff>
+    </from>
+    <to>
+      <col>11</col>
+      <colOff>30566</colOff>
+      <row>15</row>
+      <rowOff>79377</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Picture 1" descr="Obsah obrázku kruh&#10;&#10;Popis byl vytvořen automaticky"/>
+        <cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1" noChangeArrowheads="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr bwMode="auto">
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="4867277" y="3409950"/>
+          <a:ext cx="459189" cy="431802"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>14</col>
+      <colOff>114302</colOff>
+      <row>12</row>
+      <rowOff>47343</rowOff>
+    </from>
+    <to>
+      <col>16</col>
+      <colOff>40821</colOff>
+      <row>15</row>
+      <rowOff>79377</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Picture 2" descr="Obsah obrázku kruh&#10;&#10;Popis byl vytvořen automaticky"/>
+        <cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1" noChangeArrowheads="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr bwMode="auto">
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="6419852" y="3409668"/>
+          <a:ext cx="459919" cy="432084"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>19</col>
+      <colOff>114302</colOff>
+      <row>12</row>
+      <rowOff>38099</rowOff>
+    </from>
+    <to>
+      <col>21</col>
+      <colOff>18597</colOff>
+      <row>15</row>
+      <rowOff>88900</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Picture 3" descr="Obsah obrázku kruh, snímek obrazovky&#10;&#10;Popis byl vytvořen automaticky"/>
+        <cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1" noChangeArrowheads="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr bwMode="auto">
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="7905752" y="3400424"/>
+          <a:ext cx="437695" cy="450851"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>24</col>
+      <colOff>142876</colOff>
+      <row>12</row>
+      <rowOff>40887</rowOff>
+    </from>
+    <to>
+      <col>26</col>
+      <colOff>60777</colOff>
+      <row>15</row>
+      <rowOff>79376</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Picture 4" descr="Obsah obrázku kruh, snímek obrazovky&#10;&#10;Popis byl vytvořen automaticky"/>
+        <cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1" noChangeArrowheads="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr bwMode="auto">
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="9420226" y="3403212"/>
+          <a:ext cx="451301" cy="438539"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>29</col>
+      <colOff>114302</colOff>
+      <row>12</row>
+      <rowOff>38701</rowOff>
+    </from>
+    <to>
+      <col>31</col>
+      <colOff>57604</colOff>
+      <row>15</row>
+      <rowOff>74131</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Picture 5" descr="Obsah obrázku kruh&#10;&#10;Popis byl vytvořen automaticky"/>
+        <cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1" noChangeArrowheads="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr bwMode="auto">
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="10858502" y="3401026"/>
+          <a:ext cx="476702" cy="435480"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>31</col>
+      <colOff>30616</colOff>
+      <row>35</row>
+      <rowOff>53215</rowOff>
+    </from>
+    <to>
+      <col>37</col>
+      <colOff>392907</colOff>
+      <row>40</row>
+      <rowOff>125970</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="7" name="Obrázek 6" descr="Obsah obrázku text, Písmo, Grafika, logo&#10;&#10;Popis byl vytvořen automaticky"/>
+        <cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="11308216" y="9244840"/>
+          <a:ext cx="2448266" cy="1263380"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>31</col>
+      <colOff>12021</colOff>
+      <row>15</row>
+      <rowOff>656834</rowOff>
+    </from>
+    <to>
+      <col>32</col>
+      <colOff>1120323</colOff>
+      <row>17</row>
+      <rowOff>411567</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 6" descr="Obsah obrázku Písmo, Grafika, grafický design, logo&#10;&#10;Popis byl vytvořen automaticky"/>
+        <cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="22252896" y="11582009"/>
+          <a:ext cx="3041877" cy="1412083"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
 </wsDr>
 </file>
 
@@ -13799,4 +14221,2120 @@
   <pageSetup orientation="portrait" paperSize="9" scale="51" fitToHeight="0"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FFFFC000"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:AL35"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="32.28515625" defaultRowHeight="18.75"/>
+  <cols>
+    <col width="2.7109375" customWidth="1" style="1" min="1" max="1"/>
+    <col width="31.28515625" bestFit="1" customWidth="1" style="119" min="2" max="2"/>
+    <col width="31.5703125" bestFit="1" customWidth="1" style="119" min="3" max="3"/>
+    <col hidden="1" width="5.5703125" customWidth="1" style="1" min="4" max="5"/>
+    <col hidden="1" width="4.42578125" customWidth="1" style="1" min="6" max="6"/>
+    <col hidden="1" width="5.5703125" customWidth="1" style="1" min="7" max="8"/>
+    <col width="5.5703125" bestFit="1" customWidth="1" style="1" min="9" max="9"/>
+    <col width="4.28515625" customWidth="1" style="1" min="10" max="10"/>
+    <col width="4" bestFit="1" customWidth="1" style="1" min="11" max="12"/>
+    <col width="4.85546875" customWidth="1" style="1" min="13" max="13"/>
+    <col width="6.28515625" bestFit="1" customWidth="1" style="1" min="14" max="14"/>
+    <col width="4" bestFit="1" customWidth="1" style="1" min="15" max="18"/>
+    <col width="6.28515625" bestFit="1" customWidth="1" style="1" min="19" max="19"/>
+    <col width="4" bestFit="1" customWidth="1" style="1" min="20" max="23"/>
+    <col width="6.28515625" bestFit="1" customWidth="1" style="1" min="24" max="24"/>
+    <col width="4" bestFit="1" customWidth="1" style="1" min="25" max="26"/>
+    <col width="3.7109375" customWidth="1" style="1" min="27" max="27"/>
+    <col width="4" bestFit="1" customWidth="1" style="1" min="28" max="28"/>
+    <col width="6.28515625" bestFit="1" customWidth="1" style="1" min="29" max="29"/>
+    <col width="4" bestFit="1" customWidth="1" style="1" min="30" max="33"/>
+    <col width="6.28515625" bestFit="1" customWidth="1" style="1" min="34" max="34"/>
+    <col width="1.7109375" customWidth="1" style="1" min="35" max="35"/>
+    <col width="6.7109375" customWidth="1" style="1" min="36" max="36"/>
+    <col width="8.5703125" customWidth="1" style="388" min="37" max="37"/>
+    <col width="7.5703125" customWidth="1" style="120" min="38" max="38"/>
+    <col width="2.28515625" customWidth="1" style="1" min="39" max="39"/>
+    <col width="32.28515625" customWidth="1" style="1" min="40" max="16384"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="9.75" customHeight="1" thickBot="1"/>
+    <row r="2" ht="54.6" customHeight="1" thickBot="1" thickTop="1">
+      <c r="B2" s="686" t="inlineStr">
+        <is>
+          <t>FEMININES - WOMEN /  TIR DE PRECISION - SHOOTING</t>
+        </is>
+      </c>
+      <c r="C2" s="687" t="n"/>
+      <c r="D2" s="687" t="n"/>
+      <c r="E2" s="687" t="n"/>
+      <c r="F2" s="687" t="n"/>
+      <c r="G2" s="687" t="n"/>
+      <c r="H2" s="687" t="n"/>
+      <c r="I2" s="687" t="n"/>
+      <c r="J2" s="687" t="n"/>
+      <c r="K2" s="687" t="n"/>
+      <c r="L2" s="687" t="n"/>
+      <c r="M2" s="687" t="n"/>
+      <c r="N2" s="687" t="n"/>
+      <c r="O2" s="687" t="n"/>
+      <c r="P2" s="687" t="n"/>
+      <c r="Q2" s="687" t="n"/>
+      <c r="R2" s="687" t="n"/>
+      <c r="S2" s="687" t="n"/>
+      <c r="T2" s="687" t="n"/>
+      <c r="U2" s="687" t="n"/>
+      <c r="V2" s="687" t="n"/>
+      <c r="W2" s="687" t="n"/>
+      <c r="X2" s="687" t="n"/>
+      <c r="Y2" s="687" t="n"/>
+      <c r="Z2" s="687" t="n"/>
+      <c r="AA2" s="687" t="n"/>
+      <c r="AB2" s="687" t="n"/>
+      <c r="AC2" s="687" t="n"/>
+      <c r="AD2" s="687" t="n"/>
+      <c r="AE2" s="687" t="n"/>
+      <c r="AF2" s="687" t="n"/>
+      <c r="AG2" s="687" t="n"/>
+      <c r="AH2" s="687" t="n"/>
+      <c r="AI2" s="687" t="n"/>
+      <c r="AJ2" s="688" t="n"/>
+      <c r="AK2" s="392" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="AL2" s="393" t="inlineStr">
+        <is>
+          <t>Place</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28.5" customHeight="1" thickTop="1">
+      <c r="B3" s="394" t="n"/>
+      <c r="C3" s="395" t="n"/>
+      <c r="D3" s="689" t="inlineStr">
+        <is>
+          <t>Qualifiés pour les 1/4 de finales
+Qualified to 1/4 final</t>
+        </is>
+      </c>
+      <c r="E3" s="676" t="n"/>
+      <c r="F3" s="676" t="n"/>
+      <c r="G3" s="676" t="n"/>
+      <c r="H3" s="676" t="n"/>
+      <c r="I3" s="676" t="n"/>
+      <c r="J3" s="676" t="n"/>
+      <c r="K3" s="676" t="n"/>
+      <c r="L3" s="676" t="n"/>
+      <c r="M3" s="676" t="n"/>
+      <c r="N3" s="676" t="n"/>
+      <c r="O3" s="676" t="n"/>
+      <c r="P3" s="676" t="n"/>
+      <c r="Q3" s="676" t="n"/>
+      <c r="R3" s="676" t="n"/>
+      <c r="S3" s="676" t="n"/>
+      <c r="T3" s="676" t="n"/>
+      <c r="U3" s="676" t="n"/>
+      <c r="V3" s="676" t="n"/>
+      <c r="W3" s="676" t="n"/>
+      <c r="X3" s="676" t="n"/>
+      <c r="Y3" s="676" t="n"/>
+      <c r="Z3" s="676" t="n"/>
+      <c r="AA3" s="676" t="n"/>
+      <c r="AB3" s="676" t="n"/>
+      <c r="AC3" s="676" t="n"/>
+      <c r="AD3" s="676" t="n"/>
+      <c r="AE3" s="676" t="n"/>
+      <c r="AF3" s="676" t="n"/>
+      <c r="AG3" s="676" t="n"/>
+      <c r="AH3" s="676" t="n"/>
+      <c r="AI3" s="676" t="n"/>
+      <c r="AJ3" s="670" t="n"/>
+      <c r="AK3" s="399" t="n"/>
+      <c r="AL3" s="400" t="n"/>
+    </row>
+    <row r="4" ht="28.5" customHeight="1">
+      <c r="B4" s="401" t="n"/>
+      <c r="C4" s="395" t="n"/>
+      <c r="D4" s="690" t="n"/>
+      <c r="E4" s="676" t="n"/>
+      <c r="F4" s="676" t="n"/>
+      <c r="G4" s="676" t="n"/>
+      <c r="H4" s="676" t="n"/>
+      <c r="I4" s="676" t="n"/>
+      <c r="J4" s="676" t="n"/>
+      <c r="K4" s="676" t="n"/>
+      <c r="L4" s="676" t="n"/>
+      <c r="M4" s="676" t="n"/>
+      <c r="N4" s="676" t="n"/>
+      <c r="O4" s="676" t="n"/>
+      <c r="P4" s="676" t="n"/>
+      <c r="Q4" s="676" t="n"/>
+      <c r="R4" s="676" t="n"/>
+      <c r="S4" s="676" t="n"/>
+      <c r="T4" s="676" t="n"/>
+      <c r="U4" s="676" t="n"/>
+      <c r="V4" s="676" t="n"/>
+      <c r="W4" s="676" t="n"/>
+      <c r="X4" s="676" t="n"/>
+      <c r="Y4" s="676" t="n"/>
+      <c r="Z4" s="676" t="n"/>
+      <c r="AA4" s="676" t="n"/>
+      <c r="AB4" s="676" t="n"/>
+      <c r="AC4" s="676" t="n"/>
+      <c r="AD4" s="676" t="n"/>
+      <c r="AE4" s="676" t="n"/>
+      <c r="AF4" s="676" t="n"/>
+      <c r="AG4" s="676" t="n"/>
+      <c r="AH4" s="676" t="n"/>
+      <c r="AI4" s="676" t="n"/>
+      <c r="AJ4" s="670" t="n"/>
+      <c r="AK4" s="399" t="n"/>
+      <c r="AL4" s="402" t="n"/>
+    </row>
+    <row r="5" ht="28.5" customHeight="1">
+      <c r="B5" s="401" t="n"/>
+      <c r="C5" s="395" t="n"/>
+      <c r="D5" s="690" t="n"/>
+      <c r="E5" s="676" t="n"/>
+      <c r="F5" s="676" t="n"/>
+      <c r="G5" s="676" t="n"/>
+      <c r="H5" s="676" t="n"/>
+      <c r="I5" s="676" t="n"/>
+      <c r="J5" s="676" t="n"/>
+      <c r="K5" s="676" t="n"/>
+      <c r="L5" s="676" t="n"/>
+      <c r="M5" s="676" t="n"/>
+      <c r="N5" s="676" t="n"/>
+      <c r="O5" s="676" t="n"/>
+      <c r="P5" s="676" t="n"/>
+      <c r="Q5" s="676" t="n"/>
+      <c r="R5" s="676" t="n"/>
+      <c r="S5" s="676" t="n"/>
+      <c r="T5" s="676" t="n"/>
+      <c r="U5" s="676" t="n"/>
+      <c r="V5" s="676" t="n"/>
+      <c r="W5" s="676" t="n"/>
+      <c r="X5" s="676" t="n"/>
+      <c r="Y5" s="676" t="n"/>
+      <c r="Z5" s="676" t="n"/>
+      <c r="AA5" s="676" t="n"/>
+      <c r="AB5" s="676" t="n"/>
+      <c r="AC5" s="676" t="n"/>
+      <c r="AD5" s="676" t="n"/>
+      <c r="AE5" s="676" t="n"/>
+      <c r="AF5" s="676" t="n"/>
+      <c r="AG5" s="676" t="n"/>
+      <c r="AH5" s="676" t="n"/>
+      <c r="AI5" s="676" t="n"/>
+      <c r="AJ5" s="670" t="n"/>
+      <c r="AK5" s="399" t="n"/>
+      <c r="AL5" s="402" t="n"/>
+    </row>
+    <row r="6" ht="28.5" customHeight="1" thickBot="1">
+      <c r="B6" s="403" t="n"/>
+      <c r="C6" s="404" t="n"/>
+      <c r="D6" s="691" t="n"/>
+      <c r="E6" s="692" t="n"/>
+      <c r="F6" s="692" t="n"/>
+      <c r="G6" s="692" t="n"/>
+      <c r="H6" s="692" t="n"/>
+      <c r="I6" s="692" t="n"/>
+      <c r="J6" s="692" t="n"/>
+      <c r="K6" s="692" t="n"/>
+      <c r="L6" s="692" t="n"/>
+      <c r="M6" s="692" t="n"/>
+      <c r="N6" s="692" t="n"/>
+      <c r="O6" s="692" t="n"/>
+      <c r="P6" s="692" t="n"/>
+      <c r="Q6" s="692" t="n"/>
+      <c r="R6" s="692" t="n"/>
+      <c r="S6" s="692" t="n"/>
+      <c r="T6" s="692" t="n"/>
+      <c r="U6" s="692" t="n"/>
+      <c r="V6" s="692" t="n"/>
+      <c r="W6" s="692" t="n"/>
+      <c r="X6" s="692" t="n"/>
+      <c r="Y6" s="692" t="n"/>
+      <c r="Z6" s="692" t="n"/>
+      <c r="AA6" s="692" t="n"/>
+      <c r="AB6" s="692" t="n"/>
+      <c r="AC6" s="692" t="n"/>
+      <c r="AD6" s="692" t="n"/>
+      <c r="AE6" s="692" t="n"/>
+      <c r="AF6" s="692" t="n"/>
+      <c r="AG6" s="692" t="n"/>
+      <c r="AH6" s="692" t="n"/>
+      <c r="AI6" s="692" t="n"/>
+      <c r="AJ6" s="693" t="n"/>
+      <c r="AK6" s="408" t="n"/>
+      <c r="AL6" s="409" t="n"/>
+    </row>
+    <row r="7" hidden="1" ht="9.75" customFormat="1" customHeight="1" s="416" thickBot="1" thickTop="1">
+      <c r="B7" s="410" t="n"/>
+      <c r="C7" s="411" t="n"/>
+      <c r="D7" s="412" t="n"/>
+      <c r="E7" s="413" t="n"/>
+      <c r="F7" s="413" t="n"/>
+      <c r="G7" s="413" t="n"/>
+      <c r="H7" s="413" t="n"/>
+      <c r="I7" s="413" t="n"/>
+      <c r="J7" s="413" t="n"/>
+      <c r="K7" s="413" t="n"/>
+      <c r="L7" s="413" t="n"/>
+      <c r="M7" s="413" t="n"/>
+      <c r="N7" s="413" t="n"/>
+      <c r="O7" s="413" t="n"/>
+      <c r="P7" s="413" t="n"/>
+      <c r="Q7" s="413" t="n"/>
+      <c r="R7" s="413" t="n"/>
+      <c r="S7" s="413" t="n"/>
+      <c r="T7" s="413" t="n"/>
+      <c r="U7" s="413" t="n"/>
+      <c r="V7" s="413" t="n"/>
+      <c r="W7" s="413" t="n"/>
+      <c r="X7" s="413" t="n"/>
+      <c r="Y7" s="413" t="n"/>
+      <c r="Z7" s="413" t="n"/>
+      <c r="AA7" s="413" t="n"/>
+      <c r="AB7" s="413" t="n"/>
+      <c r="AC7" s="413" t="n"/>
+      <c r="AD7" s="413" t="n"/>
+      <c r="AE7" s="413" t="n"/>
+      <c r="AF7" s="413" t="n"/>
+      <c r="AG7" s="413" t="n"/>
+      <c r="AH7" s="413" t="n"/>
+      <c r="AI7" s="413" t="n"/>
+      <c r="AJ7" s="413" t="n"/>
+      <c r="AK7" s="414" t="n"/>
+      <c r="AL7" s="415" t="n"/>
+    </row>
+    <row r="8" hidden="1" ht="21.75" customHeight="1" thickBot="1">
+      <c r="B8" s="417" t="n"/>
+      <c r="C8" s="420" t="n"/>
+      <c r="D8" s="694" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Le tireur dans la repechage garde ses points de 1er tour. </t>
+        </is>
+      </c>
+      <c r="E8" s="676" t="n"/>
+      <c r="F8" s="676" t="n"/>
+      <c r="G8" s="676" t="n"/>
+      <c r="H8" s="676" t="n"/>
+      <c r="I8" s="676" t="n"/>
+      <c r="J8" s="676" t="n"/>
+      <c r="K8" s="676" t="n"/>
+      <c r="L8" s="676" t="n"/>
+      <c r="M8" s="676" t="n"/>
+      <c r="N8" s="676" t="n"/>
+      <c r="O8" s="676" t="n"/>
+      <c r="P8" s="676" t="n"/>
+      <c r="Q8" s="676" t="n"/>
+      <c r="R8" s="676" t="n"/>
+      <c r="S8" s="676" t="n"/>
+      <c r="T8" s="676" t="n"/>
+      <c r="U8" s="676" t="n"/>
+      <c r="V8" s="676" t="n"/>
+      <c r="W8" s="676" t="n"/>
+      <c r="X8" s="676" t="n"/>
+      <c r="Y8" s="676" t="n"/>
+      <c r="Z8" s="676" t="n"/>
+      <c r="AA8" s="676" t="n"/>
+      <c r="AB8" s="676" t="n"/>
+      <c r="AC8" s="676" t="n"/>
+      <c r="AD8" s="676" t="n"/>
+      <c r="AE8" s="676" t="n"/>
+      <c r="AF8" s="676" t="n"/>
+      <c r="AG8" s="676" t="n"/>
+      <c r="AH8" s="676" t="n"/>
+      <c r="AI8" s="676" t="n"/>
+      <c r="AJ8" s="676" t="n"/>
+      <c r="AK8" s="676" t="n"/>
+      <c r="AL8" s="695" t="n"/>
+    </row>
+    <row r="9" hidden="1" ht="21.75" customHeight="1" thickBot="1">
+      <c r="B9" s="422" t="n"/>
+      <c r="C9" s="420" t="n"/>
+      <c r="D9" s="694" t="inlineStr">
+        <is>
+          <t>The shooter in the repechage keeps his points of 1st round.</t>
+        </is>
+      </c>
+      <c r="E9" s="676" t="n"/>
+      <c r="F9" s="676" t="n"/>
+      <c r="G9" s="676" t="n"/>
+      <c r="H9" s="676" t="n"/>
+      <c r="I9" s="676" t="n"/>
+      <c r="J9" s="676" t="n"/>
+      <c r="K9" s="676" t="n"/>
+      <c r="L9" s="676" t="n"/>
+      <c r="M9" s="676" t="n"/>
+      <c r="N9" s="676" t="n"/>
+      <c r="O9" s="676" t="n"/>
+      <c r="P9" s="676" t="n"/>
+      <c r="Q9" s="676" t="n"/>
+      <c r="R9" s="676" t="n"/>
+      <c r="S9" s="676" t="n"/>
+      <c r="T9" s="676" t="n"/>
+      <c r="U9" s="676" t="n"/>
+      <c r="V9" s="676" t="n"/>
+      <c r="W9" s="676" t="n"/>
+      <c r="X9" s="676" t="n"/>
+      <c r="Y9" s="676" t="n"/>
+      <c r="Z9" s="676" t="n"/>
+      <c r="AA9" s="676" t="n"/>
+      <c r="AB9" s="676" t="n"/>
+      <c r="AC9" s="676" t="n"/>
+      <c r="AD9" s="676" t="n"/>
+      <c r="AE9" s="676" t="n"/>
+      <c r="AF9" s="676" t="n"/>
+      <c r="AG9" s="676" t="n"/>
+      <c r="AH9" s="676" t="n"/>
+      <c r="AI9" s="676" t="n"/>
+      <c r="AJ9" s="676" t="n"/>
+      <c r="AK9" s="676" t="n"/>
+      <c r="AL9" s="695" t="n"/>
+    </row>
+    <row r="10" ht="45" customHeight="1" thickBot="1">
+      <c r="B10" s="423" t="n"/>
+      <c r="C10" s="424" t="n"/>
+      <c r="D10" s="424" t="n"/>
+      <c r="E10" s="424" t="n"/>
+      <c r="F10" s="424" t="n"/>
+      <c r="G10" s="424" t="n"/>
+      <c r="H10" s="424" t="n"/>
+      <c r="I10" s="424" t="n"/>
+      <c r="J10" s="424" t="n"/>
+      <c r="K10" s="424" t="n"/>
+      <c r="L10" s="424" t="n"/>
+      <c r="M10" s="424" t="n"/>
+      <c r="N10" s="424" t="n"/>
+      <c r="O10" s="424" t="n"/>
+      <c r="P10" s="424" t="n"/>
+      <c r="Q10" s="424" t="n"/>
+      <c r="R10" s="424" t="n"/>
+      <c r="S10" s="424" t="n"/>
+      <c r="T10" s="424" t="n"/>
+      <c r="U10" s="424" t="n"/>
+      <c r="V10" s="424" t="n"/>
+      <c r="W10" s="424" t="n"/>
+      <c r="X10" s="424" t="n"/>
+      <c r="Y10" s="424" t="n"/>
+      <c r="Z10" s="424" t="n"/>
+      <c r="AA10" s="424" t="n"/>
+      <c r="AB10" s="424" t="n"/>
+      <c r="AC10" s="424" t="n"/>
+      <c r="AD10" s="424" t="n"/>
+      <c r="AE10" s="424" t="n"/>
+      <c r="AF10" s="424" t="n"/>
+      <c r="AG10" s="424" t="n"/>
+      <c r="AH10" s="424" t="n"/>
+      <c r="AI10" s="424" t="n"/>
+      <c r="AJ10" s="424" t="n"/>
+      <c r="AK10" s="424" t="n"/>
+      <c r="AL10" s="425" t="n"/>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="B11" s="696" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REPECHAGE DE TIR DE PRECISION
+Le tireur dans la repéchage garde ses points du 1er tour.
+The shooter in the repechage keeps his points of 1st round. </t>
+        </is>
+      </c>
+      <c r="C11" s="697" t="n"/>
+      <c r="D11" s="697" t="n"/>
+      <c r="E11" s="697" t="n"/>
+      <c r="F11" s="697" t="n"/>
+      <c r="G11" s="697" t="n"/>
+      <c r="H11" s="697" t="n"/>
+      <c r="I11" s="428" t="n"/>
+      <c r="J11" s="430" t="inlineStr">
+        <is>
+          <t>Atelier 1</t>
+        </is>
+      </c>
+      <c r="K11" s="698" t="n"/>
+      <c r="L11" s="698" t="n"/>
+      <c r="M11" s="698" t="n"/>
+      <c r="N11" s="699" t="n"/>
+      <c r="O11" s="700" t="inlineStr">
+        <is>
+          <t>Atelier 2</t>
+        </is>
+      </c>
+      <c r="P11" s="698" t="n"/>
+      <c r="Q11" s="698" t="n"/>
+      <c r="R11" s="698" t="n"/>
+      <c r="S11" s="699" t="n"/>
+      <c r="T11" s="700" t="inlineStr">
+        <is>
+          <t>Atelier 3</t>
+        </is>
+      </c>
+      <c r="U11" s="698" t="n"/>
+      <c r="V11" s="698" t="n"/>
+      <c r="W11" s="698" t="n"/>
+      <c r="X11" s="699" t="n"/>
+      <c r="Y11" s="700" t="inlineStr">
+        <is>
+          <t>Atelier 4</t>
+        </is>
+      </c>
+      <c r="Z11" s="698" t="n"/>
+      <c r="AA11" s="698" t="n"/>
+      <c r="AB11" s="698" t="n"/>
+      <c r="AC11" s="699" t="n"/>
+      <c r="AD11" s="700" t="inlineStr">
+        <is>
+          <t>Atelier 5</t>
+        </is>
+      </c>
+      <c r="AE11" s="698" t="n"/>
+      <c r="AF11" s="698" t="n"/>
+      <c r="AG11" s="698" t="n"/>
+      <c r="AH11" s="699" t="n"/>
+      <c r="AI11" s="701" t="inlineStr">
+        <is>
+          <t>REPECHAGE</t>
+        </is>
+      </c>
+      <c r="AJ11" s="702" t="n"/>
+      <c r="AK11" s="703" t="inlineStr">
+        <is>
+          <t>CUMULE</t>
+        </is>
+      </c>
+      <c r="AL11" s="704" t="inlineStr">
+        <is>
+          <t>Classement</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="B12" s="705" t="n"/>
+      <c r="I12" s="437" t="n"/>
+      <c r="J12" s="439" t="inlineStr">
+        <is>
+          <t>Boule seule</t>
+        </is>
+      </c>
+      <c r="K12" s="706" t="n"/>
+      <c r="L12" s="706" t="n"/>
+      <c r="M12" s="706" t="n"/>
+      <c r="N12" s="707" t="n"/>
+      <c r="O12" s="708" t="inlineStr">
+        <is>
+          <t>Boule derrière but</t>
+        </is>
+      </c>
+      <c r="P12" s="706" t="n"/>
+      <c r="Q12" s="706" t="n"/>
+      <c r="R12" s="706" t="n"/>
+      <c r="S12" s="707" t="n"/>
+      <c r="T12" s="708" t="inlineStr">
+        <is>
+          <t>Entre deux boules</t>
+        </is>
+      </c>
+      <c r="U12" s="706" t="n"/>
+      <c r="V12" s="706" t="n"/>
+      <c r="W12" s="706" t="n"/>
+      <c r="X12" s="707" t="n"/>
+      <c r="Y12" s="708" t="inlineStr">
+        <is>
+          <t>Sautée</t>
+        </is>
+      </c>
+      <c r="Z12" s="706" t="n"/>
+      <c r="AA12" s="706" t="n"/>
+      <c r="AB12" s="706" t="n"/>
+      <c r="AC12" s="707" t="n"/>
+      <c r="AD12" s="708" t="inlineStr">
+        <is>
+          <t>But</t>
+        </is>
+      </c>
+      <c r="AE12" s="706" t="n"/>
+      <c r="AF12" s="706" t="n"/>
+      <c r="AG12" s="706" t="n"/>
+      <c r="AH12" s="707" t="n"/>
+      <c r="AI12" s="690" t="n"/>
+      <c r="AJ12" s="670" t="n"/>
+      <c r="AK12" s="709" t="n"/>
+      <c r="AL12" s="709" t="n"/>
+    </row>
+    <row r="13" ht="10.5" customHeight="1">
+      <c r="B13" s="705" t="n"/>
+      <c r="I13" s="437" t="n"/>
+      <c r="J13" s="445" t="inlineStr">
+        <is>
+          <t>Carreau: 5 p</t>
+        </is>
+      </c>
+      <c r="K13" s="710" t="n"/>
+      <c r="L13" s="710" t="n"/>
+      <c r="M13" s="710" t="n"/>
+      <c r="N13" s="711" t="n"/>
+      <c r="O13" s="712" t="inlineStr">
+        <is>
+          <t>Carreau: 5 p</t>
+        </is>
+      </c>
+      <c r="P13" s="710" t="n"/>
+      <c r="Q13" s="710" t="n"/>
+      <c r="R13" s="710" t="n"/>
+      <c r="S13" s="711" t="n"/>
+      <c r="T13" s="712" t="inlineStr">
+        <is>
+          <t>Carreau: 5 p</t>
+        </is>
+      </c>
+      <c r="U13" s="710" t="n"/>
+      <c r="V13" s="710" t="n"/>
+      <c r="W13" s="710" t="n"/>
+      <c r="X13" s="711" t="n"/>
+      <c r="Y13" s="712" t="inlineStr">
+        <is>
+          <t>Carreau: 5 p</t>
+        </is>
+      </c>
+      <c r="Z13" s="710" t="n"/>
+      <c r="AA13" s="710" t="n"/>
+      <c r="AB13" s="710" t="n"/>
+      <c r="AC13" s="711" t="n"/>
+      <c r="AD13" s="712" t="inlineStr">
+        <is>
+          <t>Carreau: 5 p</t>
+        </is>
+      </c>
+      <c r="AE13" s="710" t="n"/>
+      <c r="AF13" s="710" t="n"/>
+      <c r="AG13" s="710" t="n"/>
+      <c r="AH13" s="711" t="n"/>
+      <c r="AI13" s="690" t="n"/>
+      <c r="AJ13" s="670" t="n"/>
+      <c r="AK13" s="709" t="n"/>
+      <c r="AL13" s="709" t="n"/>
+    </row>
+    <row r="14" ht="10.5" customHeight="1">
+      <c r="B14" s="705" t="n"/>
+      <c r="I14" s="447" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="J14" s="449" t="inlineStr">
+        <is>
+          <t>Réussi: 3 p</t>
+        </is>
+      </c>
+      <c r="N14" s="713" t="n"/>
+      <c r="O14" s="714" t="inlineStr">
+        <is>
+          <t>Réussi: 3 p</t>
+        </is>
+      </c>
+      <c r="S14" s="713" t="n"/>
+      <c r="T14" s="714" t="inlineStr">
+        <is>
+          <t>Réussi: 3 p</t>
+        </is>
+      </c>
+      <c r="X14" s="713" t="n"/>
+      <c r="Y14" s="714" t="inlineStr">
+        <is>
+          <t>Réussi: 3 p</t>
+        </is>
+      </c>
+      <c r="AC14" s="713" t="n"/>
+      <c r="AD14" s="714" t="inlineStr">
+        <is>
+          <t>Touché: 3 p</t>
+        </is>
+      </c>
+      <c r="AH14" s="713" t="n"/>
+      <c r="AI14" s="690" t="n"/>
+      <c r="AJ14" s="670" t="n"/>
+      <c r="AK14" s="709" t="n"/>
+      <c r="AL14" s="709" t="n"/>
+    </row>
+    <row r="15" ht="10.5" customHeight="1">
+      <c r="B15" s="705" t="n"/>
+      <c r="I15" s="715" t="n"/>
+      <c r="J15" s="449" t="inlineStr">
+        <is>
+          <t>Touché: 1 p</t>
+        </is>
+      </c>
+      <c r="N15" s="713" t="n"/>
+      <c r="O15" s="714" t="inlineStr">
+        <is>
+          <t>Touché: 1 p</t>
+        </is>
+      </c>
+      <c r="S15" s="713" t="n"/>
+      <c r="T15" s="714" t="inlineStr">
+        <is>
+          <t>Touché: 1 p</t>
+        </is>
+      </c>
+      <c r="X15" s="713" t="n"/>
+      <c r="Y15" s="714" t="inlineStr">
+        <is>
+          <t>Touché: 1 p</t>
+        </is>
+      </c>
+      <c r="AC15" s="713" t="n"/>
+      <c r="AD15" s="714" t="n"/>
+      <c r="AH15" s="713" t="n"/>
+      <c r="AI15" s="690" t="n"/>
+      <c r="AJ15" s="670" t="n"/>
+      <c r="AK15" s="709" t="n"/>
+      <c r="AL15" s="709" t="n"/>
+    </row>
+    <row r="16" ht="10.5" customHeight="1">
+      <c r="B16" s="705" t="n"/>
+      <c r="I16" s="715" t="n"/>
+      <c r="J16" s="453" t="inlineStr">
+        <is>
+          <t>Manqué: 0 p</t>
+        </is>
+      </c>
+      <c r="K16" s="716" t="n"/>
+      <c r="L16" s="716" t="n"/>
+      <c r="M16" s="716" t="n"/>
+      <c r="N16" s="717" t="n"/>
+      <c r="O16" s="718" t="inlineStr">
+        <is>
+          <t>Manqué: 0 p</t>
+        </is>
+      </c>
+      <c r="P16" s="716" t="n"/>
+      <c r="Q16" s="716" t="n"/>
+      <c r="R16" s="716" t="n"/>
+      <c r="S16" s="717" t="n"/>
+      <c r="T16" s="718" t="inlineStr">
+        <is>
+          <t>Manqué: 0 p</t>
+        </is>
+      </c>
+      <c r="U16" s="716" t="n"/>
+      <c r="V16" s="716" t="n"/>
+      <c r="W16" s="716" t="n"/>
+      <c r="X16" s="717" t="n"/>
+      <c r="Y16" s="718" t="inlineStr">
+        <is>
+          <t>Manqué: 0 p</t>
+        </is>
+      </c>
+      <c r="Z16" s="716" t="n"/>
+      <c r="AA16" s="716" t="n"/>
+      <c r="AB16" s="716" t="n"/>
+      <c r="AC16" s="717" t="n"/>
+      <c r="AD16" s="718" t="inlineStr">
+        <is>
+          <t>Manqué: 0 p</t>
+        </is>
+      </c>
+      <c r="AE16" s="716" t="n"/>
+      <c r="AF16" s="716" t="n"/>
+      <c r="AG16" s="716" t="n"/>
+      <c r="AH16" s="717" t="n"/>
+      <c r="AI16" s="690" t="n"/>
+      <c r="AJ16" s="670" t="n"/>
+      <c r="AK16" s="709" t="n"/>
+      <c r="AL16" s="709" t="n"/>
+    </row>
+    <row r="17" ht="27" customHeight="1" thickBot="1">
+      <c r="B17" s="719" t="n"/>
+      <c r="C17" s="720" t="n"/>
+      <c r="D17" s="720" t="n"/>
+      <c r="E17" s="720" t="n"/>
+      <c r="F17" s="720" t="n"/>
+      <c r="G17" s="720" t="n"/>
+      <c r="H17" s="720" t="n"/>
+      <c r="I17" s="457" t="inlineStr">
+        <is>
+          <t>TOT</t>
+        </is>
+      </c>
+      <c r="J17" s="458" t="inlineStr">
+        <is>
+          <t>6m</t>
+        </is>
+      </c>
+      <c r="K17" s="459" t="inlineStr">
+        <is>
+          <t>7m</t>
+        </is>
+      </c>
+      <c r="L17" s="459" t="inlineStr">
+        <is>
+          <t>8m</t>
+        </is>
+      </c>
+      <c r="M17" s="459" t="inlineStr">
+        <is>
+          <t>9m</t>
+        </is>
+      </c>
+      <c r="N17" s="460" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="O17" s="461" t="inlineStr">
+        <is>
+          <t>6m</t>
+        </is>
+      </c>
+      <c r="P17" s="459" t="inlineStr">
+        <is>
+          <t>7m</t>
+        </is>
+      </c>
+      <c r="Q17" s="459" t="inlineStr">
+        <is>
+          <t>8m</t>
+        </is>
+      </c>
+      <c r="R17" s="459" t="inlineStr">
+        <is>
+          <t>9m</t>
+        </is>
+      </c>
+      <c r="S17" s="460" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="T17" s="461" t="inlineStr">
+        <is>
+          <t>6m</t>
+        </is>
+      </c>
+      <c r="U17" s="459" t="inlineStr">
+        <is>
+          <t>7m</t>
+        </is>
+      </c>
+      <c r="V17" s="459" t="inlineStr">
+        <is>
+          <t>8m</t>
+        </is>
+      </c>
+      <c r="W17" s="459" t="inlineStr">
+        <is>
+          <t>9m</t>
+        </is>
+      </c>
+      <c r="X17" s="460" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="Y17" s="461" t="inlineStr">
+        <is>
+          <t>6m</t>
+        </is>
+      </c>
+      <c r="Z17" s="459" t="inlineStr">
+        <is>
+          <t>7m</t>
+        </is>
+      </c>
+      <c r="AA17" s="459" t="inlineStr">
+        <is>
+          <t>8m</t>
+        </is>
+      </c>
+      <c r="AB17" s="459" t="inlineStr">
+        <is>
+          <t>9m</t>
+        </is>
+      </c>
+      <c r="AC17" s="460" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="AD17" s="461" t="inlineStr">
+        <is>
+          <t>6m</t>
+        </is>
+      </c>
+      <c r="AE17" s="459" t="inlineStr">
+        <is>
+          <t>7m</t>
+        </is>
+      </c>
+      <c r="AF17" s="459" t="inlineStr">
+        <is>
+          <t>8m</t>
+        </is>
+      </c>
+      <c r="AG17" s="459" t="inlineStr">
+        <is>
+          <t>9m</t>
+        </is>
+      </c>
+      <c r="AH17" s="460" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="AI17" s="721" t="n"/>
+      <c r="AJ17" s="683" t="n"/>
+      <c r="AK17" s="722" t="n"/>
+      <c r="AL17" s="722" t="n"/>
+    </row>
+    <row r="18" ht="30" customFormat="1" customHeight="1" s="477" thickTop="1">
+      <c r="B18" s="465" t="n"/>
+      <c r="C18" s="10" t="n"/>
+      <c r="D18" s="466" t="n"/>
+      <c r="E18" s="467" t="n"/>
+      <c r="F18" s="467" t="n"/>
+      <c r="G18" s="467" t="n"/>
+      <c r="H18" s="467" t="n"/>
+      <c r="I18" s="468" t="n"/>
+      <c r="J18" s="469" t="n"/>
+      <c r="K18" s="470" t="n"/>
+      <c r="L18" s="470" t="n"/>
+      <c r="M18" s="470" t="n"/>
+      <c r="N18" s="471" t="n"/>
+      <c r="O18" s="469" t="n"/>
+      <c r="P18" s="470" t="n"/>
+      <c r="Q18" s="470" t="n"/>
+      <c r="R18" s="470" t="n"/>
+      <c r="S18" s="471" t="n"/>
+      <c r="T18" s="469" t="n"/>
+      <c r="U18" s="470" t="n"/>
+      <c r="V18" s="470" t="n"/>
+      <c r="W18" s="470" t="n"/>
+      <c r="X18" s="471" t="n"/>
+      <c r="Y18" s="469" t="n"/>
+      <c r="Z18" s="470" t="n"/>
+      <c r="AA18" s="470" t="n"/>
+      <c r="AB18" s="470" t="n"/>
+      <c r="AC18" s="471" t="n"/>
+      <c r="AD18" s="472" t="n"/>
+      <c r="AE18" s="470" t="n"/>
+      <c r="AF18" s="470" t="n"/>
+      <c r="AG18" s="470" t="n"/>
+      <c r="AH18" s="471" t="n"/>
+      <c r="AI18" s="473" t="n"/>
+      <c r="AJ18" s="474" t="n"/>
+      <c r="AK18" s="475" t="n"/>
+      <c r="AL18" s="476" t="n"/>
+    </row>
+    <row r="19" ht="30" customFormat="1" customHeight="1" s="477">
+      <c r="B19" s="465" t="n"/>
+      <c r="C19" s="395" t="n"/>
+      <c r="D19" s="478" t="n"/>
+      <c r="E19" s="479" t="n"/>
+      <c r="F19" s="479" t="n"/>
+      <c r="G19" s="479" t="n"/>
+      <c r="H19" s="479" t="n"/>
+      <c r="I19" s="468" t="n"/>
+      <c r="J19" s="480" t="n"/>
+      <c r="K19" s="481" t="n"/>
+      <c r="L19" s="481" t="n"/>
+      <c r="M19" s="481" t="n"/>
+      <c r="N19" s="482" t="n"/>
+      <c r="O19" s="480" t="n"/>
+      <c r="P19" s="481" t="n"/>
+      <c r="Q19" s="481" t="n"/>
+      <c r="R19" s="481" t="n"/>
+      <c r="S19" s="482" t="n"/>
+      <c r="T19" s="480" t="n"/>
+      <c r="U19" s="481" t="n"/>
+      <c r="V19" s="481" t="n"/>
+      <c r="W19" s="481" t="n"/>
+      <c r="X19" s="482" t="n"/>
+      <c r="Y19" s="480" t="n"/>
+      <c r="Z19" s="481" t="n"/>
+      <c r="AA19" s="481" t="n"/>
+      <c r="AB19" s="481" t="n"/>
+      <c r="AC19" s="482" t="n"/>
+      <c r="AD19" s="483" t="n"/>
+      <c r="AE19" s="481" t="n"/>
+      <c r="AF19" s="481" t="n"/>
+      <c r="AG19" s="481" t="n"/>
+      <c r="AH19" s="482" t="n"/>
+      <c r="AI19" s="484" t="n"/>
+      <c r="AJ19" s="468" t="n"/>
+      <c r="AK19" s="485" t="n"/>
+      <c r="AL19" s="486" t="n"/>
+    </row>
+    <row r="20" ht="30" customFormat="1" customHeight="1" s="477">
+      <c r="B20" s="465" t="n"/>
+      <c r="C20" s="395" t="n"/>
+      <c r="D20" s="478" t="n"/>
+      <c r="E20" s="479" t="n"/>
+      <c r="F20" s="479" t="n"/>
+      <c r="G20" s="479" t="n"/>
+      <c r="H20" s="479" t="n"/>
+      <c r="I20" s="468" t="n"/>
+      <c r="J20" s="480" t="n"/>
+      <c r="K20" s="481" t="n"/>
+      <c r="L20" s="481" t="n"/>
+      <c r="M20" s="481" t="n"/>
+      <c r="N20" s="482" t="n"/>
+      <c r="O20" s="480" t="n"/>
+      <c r="P20" s="481" t="n"/>
+      <c r="Q20" s="481" t="n"/>
+      <c r="R20" s="481" t="n"/>
+      <c r="S20" s="482" t="n"/>
+      <c r="T20" s="480" t="n"/>
+      <c r="U20" s="481" t="n"/>
+      <c r="V20" s="481" t="n"/>
+      <c r="W20" s="481" t="n"/>
+      <c r="X20" s="482" t="n"/>
+      <c r="Y20" s="480" t="n"/>
+      <c r="Z20" s="481" t="n"/>
+      <c r="AA20" s="481" t="n"/>
+      <c r="AB20" s="481" t="n"/>
+      <c r="AC20" s="482" t="n"/>
+      <c r="AD20" s="483" t="n"/>
+      <c r="AE20" s="481" t="n"/>
+      <c r="AF20" s="481" t="n"/>
+      <c r="AG20" s="481" t="n"/>
+      <c r="AH20" s="482" t="n"/>
+      <c r="AI20" s="484" t="n"/>
+      <c r="AJ20" s="468" t="n"/>
+      <c r="AK20" s="485" t="n"/>
+      <c r="AL20" s="486" t="n"/>
+    </row>
+    <row r="21" ht="30" customFormat="1" customHeight="1" s="477" thickBot="1">
+      <c r="B21" s="487" t="n"/>
+      <c r="C21" s="8" t="n"/>
+      <c r="D21" s="488" t="n"/>
+      <c r="E21" s="489" t="n"/>
+      <c r="F21" s="489" t="n"/>
+      <c r="G21" s="489" t="n"/>
+      <c r="H21" s="489" t="n"/>
+      <c r="I21" s="490" t="n"/>
+      <c r="J21" s="491" t="n"/>
+      <c r="K21" s="492" t="n"/>
+      <c r="L21" s="492" t="n"/>
+      <c r="M21" s="492" t="n"/>
+      <c r="N21" s="493" t="n"/>
+      <c r="O21" s="491" t="n"/>
+      <c r="P21" s="492" t="n"/>
+      <c r="Q21" s="492" t="n"/>
+      <c r="R21" s="492" t="n"/>
+      <c r="S21" s="493" t="n"/>
+      <c r="T21" s="491" t="n"/>
+      <c r="U21" s="492" t="n"/>
+      <c r="V21" s="492" t="n"/>
+      <c r="W21" s="492" t="n"/>
+      <c r="X21" s="493" t="n"/>
+      <c r="Y21" s="491" t="n"/>
+      <c r="Z21" s="492" t="n"/>
+      <c r="AA21" s="492" t="n"/>
+      <c r="AB21" s="492" t="n"/>
+      <c r="AC21" s="493" t="n"/>
+      <c r="AD21" s="494" t="n"/>
+      <c r="AE21" s="492" t="n"/>
+      <c r="AF21" s="492" t="n"/>
+      <c r="AG21" s="492" t="n"/>
+      <c r="AH21" s="493" t="n"/>
+      <c r="AI21" s="495" t="n"/>
+      <c r="AJ21" s="490" t="n"/>
+      <c r="AK21" s="496" t="n"/>
+      <c r="AL21" s="497" t="n"/>
+    </row>
+    <row r="22" ht="30" customFormat="1" customHeight="1" s="477" thickTop="1">
+      <c r="B22" s="498" t="n"/>
+      <c r="C22" s="499" t="n"/>
+      <c r="D22" s="500" t="n"/>
+      <c r="E22" s="501" t="n"/>
+      <c r="F22" s="501" t="n"/>
+      <c r="G22" s="501" t="n"/>
+      <c r="H22" s="501" t="n"/>
+      <c r="I22" s="468" t="n"/>
+      <c r="J22" s="502" t="n"/>
+      <c r="K22" s="503" t="n"/>
+      <c r="L22" s="503" t="n"/>
+      <c r="M22" s="503" t="n"/>
+      <c r="N22" s="504" t="n"/>
+      <c r="O22" s="502" t="n"/>
+      <c r="P22" s="503" t="n"/>
+      <c r="Q22" s="503" t="n"/>
+      <c r="R22" s="503" t="n"/>
+      <c r="S22" s="504" t="n"/>
+      <c r="T22" s="502" t="n"/>
+      <c r="U22" s="503" t="n"/>
+      <c r="V22" s="503" t="n"/>
+      <c r="W22" s="503" t="n"/>
+      <c r="X22" s="504" t="n"/>
+      <c r="Y22" s="502" t="n"/>
+      <c r="Z22" s="503" t="n"/>
+      <c r="AA22" s="503" t="n"/>
+      <c r="AB22" s="503" t="n"/>
+      <c r="AC22" s="504" t="n"/>
+      <c r="AD22" s="483" t="n"/>
+      <c r="AE22" s="503" t="n"/>
+      <c r="AF22" s="503" t="n"/>
+      <c r="AG22" s="503" t="n"/>
+      <c r="AH22" s="504" t="n"/>
+      <c r="AI22" s="484" t="n"/>
+      <c r="AJ22" s="484" t="n"/>
+      <c r="AK22" s="505" t="n"/>
+      <c r="AL22" s="506" t="n"/>
+    </row>
+    <row r="23" ht="30" customFormat="1" customHeight="1" s="477">
+      <c r="B23" s="498" t="n"/>
+      <c r="C23" s="507" t="n"/>
+      <c r="D23" s="478" t="n"/>
+      <c r="E23" s="479" t="n"/>
+      <c r="F23" s="479" t="n"/>
+      <c r="G23" s="479" t="n"/>
+      <c r="H23" s="479" t="n"/>
+      <c r="I23" s="468" t="n"/>
+      <c r="J23" s="480" t="n"/>
+      <c r="K23" s="481" t="n"/>
+      <c r="L23" s="481" t="n"/>
+      <c r="M23" s="481" t="n"/>
+      <c r="N23" s="482" t="n"/>
+      <c r="O23" s="480" t="n"/>
+      <c r="P23" s="481" t="n"/>
+      <c r="Q23" s="481" t="n"/>
+      <c r="R23" s="481" t="n"/>
+      <c r="S23" s="482" t="n"/>
+      <c r="T23" s="480" t="n"/>
+      <c r="U23" s="481" t="n"/>
+      <c r="V23" s="481" t="n"/>
+      <c r="W23" s="481" t="n"/>
+      <c r="X23" s="482" t="n"/>
+      <c r="Y23" s="480" t="n"/>
+      <c r="Z23" s="481" t="n"/>
+      <c r="AA23" s="481" t="n"/>
+      <c r="AB23" s="481" t="n"/>
+      <c r="AC23" s="482" t="n"/>
+      <c r="AD23" s="483" t="n"/>
+      <c r="AE23" s="481" t="n"/>
+      <c r="AF23" s="481" t="n"/>
+      <c r="AG23" s="481" t="n"/>
+      <c r="AH23" s="482" t="n"/>
+      <c r="AI23" s="484" t="n"/>
+      <c r="AJ23" s="484" t="n"/>
+      <c r="AK23" s="505" t="n"/>
+      <c r="AL23" s="506" t="n"/>
+    </row>
+    <row r="24" ht="30" customFormat="1" customHeight="1" s="477">
+      <c r="B24" s="498" t="n"/>
+      <c r="C24" s="507" t="n"/>
+      <c r="D24" s="478" t="n"/>
+      <c r="E24" s="479" t="n"/>
+      <c r="F24" s="479" t="n"/>
+      <c r="G24" s="479" t="n"/>
+      <c r="H24" s="479" t="n"/>
+      <c r="I24" s="468" t="n"/>
+      <c r="J24" s="480" t="n"/>
+      <c r="K24" s="481" t="n"/>
+      <c r="L24" s="481" t="n"/>
+      <c r="M24" s="481" t="n"/>
+      <c r="N24" s="482" t="n"/>
+      <c r="O24" s="480" t="n"/>
+      <c r="P24" s="481" t="n"/>
+      <c r="Q24" s="481" t="n"/>
+      <c r="R24" s="481" t="n"/>
+      <c r="S24" s="482" t="n"/>
+      <c r="T24" s="480" t="n"/>
+      <c r="U24" s="481" t="n"/>
+      <c r="V24" s="481" t="n"/>
+      <c r="W24" s="481" t="n"/>
+      <c r="X24" s="482" t="n"/>
+      <c r="Y24" s="480" t="n"/>
+      <c r="Z24" s="481" t="n"/>
+      <c r="AA24" s="481" t="n"/>
+      <c r="AB24" s="481" t="n"/>
+      <c r="AC24" s="482" t="n"/>
+      <c r="AD24" s="483" t="n"/>
+      <c r="AE24" s="481" t="n"/>
+      <c r="AF24" s="481" t="n"/>
+      <c r="AG24" s="481" t="n"/>
+      <c r="AH24" s="482" t="n"/>
+      <c r="AI24" s="484" t="n"/>
+      <c r="AJ24" s="484" t="n"/>
+      <c r="AK24" s="505" t="n"/>
+      <c r="AL24" s="506" t="n"/>
+    </row>
+    <row r="25" ht="30" customFormat="1" customHeight="1" s="477">
+      <c r="B25" s="498" t="n"/>
+      <c r="C25" s="507" t="n"/>
+      <c r="D25" s="478" t="n"/>
+      <c r="E25" s="479" t="n"/>
+      <c r="F25" s="479" t="n"/>
+      <c r="G25" s="479" t="n"/>
+      <c r="H25" s="479" t="n"/>
+      <c r="I25" s="468" t="n"/>
+      <c r="J25" s="480" t="n"/>
+      <c r="K25" s="481" t="n"/>
+      <c r="L25" s="481" t="n"/>
+      <c r="M25" s="481" t="n"/>
+      <c r="N25" s="482" t="n"/>
+      <c r="O25" s="480" t="n"/>
+      <c r="P25" s="481" t="n"/>
+      <c r="Q25" s="481" t="n"/>
+      <c r="R25" s="481" t="n"/>
+      <c r="S25" s="482" t="n"/>
+      <c r="T25" s="480" t="n"/>
+      <c r="U25" s="481" t="n"/>
+      <c r="V25" s="481" t="n"/>
+      <c r="W25" s="481" t="n"/>
+      <c r="X25" s="482" t="n"/>
+      <c r="Y25" s="480" t="n"/>
+      <c r="Z25" s="481" t="n"/>
+      <c r="AA25" s="481" t="n"/>
+      <c r="AB25" s="481" t="n"/>
+      <c r="AC25" s="482" t="n"/>
+      <c r="AD25" s="483" t="n"/>
+      <c r="AE25" s="481" t="n"/>
+      <c r="AF25" s="481" t="n"/>
+      <c r="AG25" s="481" t="n"/>
+      <c r="AH25" s="482" t="n"/>
+      <c r="AI25" s="484" t="n"/>
+      <c r="AJ25" s="484" t="n"/>
+      <c r="AK25" s="505" t="n"/>
+      <c r="AL25" s="506" t="n"/>
+    </row>
+    <row r="26" ht="30" customFormat="1" customHeight="1" s="477">
+      <c r="B26" s="498" t="n"/>
+      <c r="C26" s="507" t="n"/>
+      <c r="D26" s="478" t="n"/>
+      <c r="E26" s="479" t="n"/>
+      <c r="F26" s="479" t="n"/>
+      <c r="G26" s="479" t="n"/>
+      <c r="H26" s="479" t="n"/>
+      <c r="I26" s="468" t="n"/>
+      <c r="J26" s="480" t="n"/>
+      <c r="K26" s="481" t="n"/>
+      <c r="L26" s="481" t="n"/>
+      <c r="M26" s="481" t="n"/>
+      <c r="N26" s="482" t="n"/>
+      <c r="O26" s="480" t="n"/>
+      <c r="P26" s="481" t="n"/>
+      <c r="Q26" s="481" t="n"/>
+      <c r="R26" s="481" t="n"/>
+      <c r="S26" s="482" t="n"/>
+      <c r="T26" s="480" t="n"/>
+      <c r="U26" s="481" t="n"/>
+      <c r="V26" s="481" t="n"/>
+      <c r="W26" s="481" t="n"/>
+      <c r="X26" s="482" t="n"/>
+      <c r="Y26" s="480" t="n"/>
+      <c r="Z26" s="481" t="n"/>
+      <c r="AA26" s="481" t="n"/>
+      <c r="AB26" s="481" t="n"/>
+      <c r="AC26" s="482" t="n"/>
+      <c r="AD26" s="483" t="n"/>
+      <c r="AE26" s="481" t="n"/>
+      <c r="AF26" s="481" t="n"/>
+      <c r="AG26" s="481" t="n"/>
+      <c r="AH26" s="482" t="n"/>
+      <c r="AI26" s="484" t="n"/>
+      <c r="AJ26" s="484" t="n"/>
+      <c r="AK26" s="505" t="n"/>
+      <c r="AL26" s="506" t="n"/>
+    </row>
+    <row r="27" ht="30" customFormat="1" customHeight="1" s="477">
+      <c r="B27" s="498" t="n"/>
+      <c r="C27" s="507" t="n"/>
+      <c r="D27" s="478" t="n"/>
+      <c r="E27" s="479" t="n"/>
+      <c r="F27" s="479" t="n"/>
+      <c r="G27" s="479" t="n"/>
+      <c r="H27" s="479" t="n"/>
+      <c r="I27" s="468" t="n"/>
+      <c r="J27" s="480" t="n"/>
+      <c r="K27" s="481" t="n"/>
+      <c r="L27" s="481" t="n"/>
+      <c r="M27" s="481" t="n"/>
+      <c r="N27" s="482" t="n"/>
+      <c r="O27" s="480" t="n"/>
+      <c r="P27" s="481" t="n"/>
+      <c r="Q27" s="481" t="n"/>
+      <c r="R27" s="481" t="n"/>
+      <c r="S27" s="482" t="n"/>
+      <c r="T27" s="480" t="n"/>
+      <c r="U27" s="481" t="n"/>
+      <c r="V27" s="481" t="n"/>
+      <c r="W27" s="481" t="n"/>
+      <c r="X27" s="482" t="n"/>
+      <c r="Y27" s="480" t="n"/>
+      <c r="Z27" s="481" t="n"/>
+      <c r="AA27" s="481" t="n"/>
+      <c r="AB27" s="481" t="n"/>
+      <c r="AC27" s="482" t="n"/>
+      <c r="AD27" s="483" t="n"/>
+      <c r="AE27" s="481" t="n"/>
+      <c r="AF27" s="481" t="n"/>
+      <c r="AG27" s="481" t="n"/>
+      <c r="AH27" s="482" t="n"/>
+      <c r="AI27" s="484" t="n"/>
+      <c r="AJ27" s="484" t="n"/>
+      <c r="AK27" s="505" t="n"/>
+      <c r="AL27" s="506" t="n"/>
+    </row>
+    <row r="28" ht="30" customFormat="1" customHeight="1" s="477">
+      <c r="B28" s="498" t="n"/>
+      <c r="C28" s="507" t="n"/>
+      <c r="D28" s="478" t="n"/>
+      <c r="E28" s="479" t="n"/>
+      <c r="F28" s="479" t="n"/>
+      <c r="G28" s="479" t="n"/>
+      <c r="H28" s="479" t="n"/>
+      <c r="I28" s="468" t="n"/>
+      <c r="J28" s="480" t="n"/>
+      <c r="K28" s="481" t="n"/>
+      <c r="L28" s="481" t="n"/>
+      <c r="M28" s="481" t="n"/>
+      <c r="N28" s="482" t="n"/>
+      <c r="O28" s="480" t="n"/>
+      <c r="P28" s="481" t="n"/>
+      <c r="Q28" s="481" t="n"/>
+      <c r="R28" s="481" t="n"/>
+      <c r="S28" s="482" t="n"/>
+      <c r="T28" s="480" t="n"/>
+      <c r="U28" s="481" t="n"/>
+      <c r="V28" s="481" t="n"/>
+      <c r="W28" s="481" t="n"/>
+      <c r="X28" s="482" t="n"/>
+      <c r="Y28" s="480" t="n"/>
+      <c r="Z28" s="481" t="n"/>
+      <c r="AA28" s="481" t="n"/>
+      <c r="AB28" s="481" t="n"/>
+      <c r="AC28" s="482" t="n"/>
+      <c r="AD28" s="483" t="n"/>
+      <c r="AE28" s="481" t="n"/>
+      <c r="AF28" s="481" t="n"/>
+      <c r="AG28" s="481" t="n"/>
+      <c r="AH28" s="482" t="n"/>
+      <c r="AI28" s="484" t="n"/>
+      <c r="AJ28" s="484" t="n"/>
+      <c r="AK28" s="505" t="n"/>
+      <c r="AL28" s="506" t="n"/>
+    </row>
+    <row r="29" ht="30" customFormat="1" customHeight="1" s="477">
+      <c r="B29" s="498" t="n"/>
+      <c r="C29" s="507" t="n"/>
+      <c r="D29" s="478" t="n"/>
+      <c r="E29" s="479" t="n"/>
+      <c r="F29" s="479" t="n"/>
+      <c r="G29" s="479" t="n"/>
+      <c r="H29" s="479" t="n"/>
+      <c r="I29" s="468" t="n"/>
+      <c r="J29" s="480" t="n"/>
+      <c r="K29" s="481" t="n"/>
+      <c r="L29" s="481" t="n"/>
+      <c r="M29" s="481" t="n"/>
+      <c r="N29" s="482" t="n"/>
+      <c r="O29" s="480" t="n"/>
+      <c r="P29" s="481" t="n"/>
+      <c r="Q29" s="481" t="n"/>
+      <c r="R29" s="481" t="n"/>
+      <c r="S29" s="482" t="n"/>
+      <c r="T29" s="480" t="n"/>
+      <c r="U29" s="481" t="n"/>
+      <c r="V29" s="481" t="n"/>
+      <c r="W29" s="481" t="n"/>
+      <c r="X29" s="482" t="n"/>
+      <c r="Y29" s="480" t="n"/>
+      <c r="Z29" s="481" t="n"/>
+      <c r="AA29" s="481" t="n"/>
+      <c r="AB29" s="481" t="n"/>
+      <c r="AC29" s="482" t="n"/>
+      <c r="AD29" s="483" t="n"/>
+      <c r="AE29" s="481" t="n"/>
+      <c r="AF29" s="481" t="n"/>
+      <c r="AG29" s="481" t="n"/>
+      <c r="AH29" s="482" t="n"/>
+      <c r="AI29" s="484" t="n"/>
+      <c r="AJ29" s="484" t="n"/>
+      <c r="AK29" s="505" t="n"/>
+      <c r="AL29" s="506" t="n"/>
+    </row>
+    <row r="30" ht="30" customFormat="1" customHeight="1" s="477" thickBot="1">
+      <c r="B30" s="508" t="n"/>
+      <c r="C30" s="509" t="n"/>
+      <c r="D30" s="510" t="n"/>
+      <c r="E30" s="511" t="n"/>
+      <c r="F30" s="511" t="n"/>
+      <c r="G30" s="511" t="n"/>
+      <c r="H30" s="511" t="n"/>
+      <c r="I30" s="512" t="n"/>
+      <c r="J30" s="513" t="n"/>
+      <c r="K30" s="514" t="n"/>
+      <c r="L30" s="514" t="n"/>
+      <c r="M30" s="514" t="n"/>
+      <c r="N30" s="515" t="n"/>
+      <c r="O30" s="513" t="n"/>
+      <c r="P30" s="514" t="n"/>
+      <c r="Q30" s="514" t="n"/>
+      <c r="R30" s="514" t="n"/>
+      <c r="S30" s="515" t="n"/>
+      <c r="T30" s="513" t="n"/>
+      <c r="U30" s="514" t="n"/>
+      <c r="V30" s="514" t="n"/>
+      <c r="W30" s="514" t="n"/>
+      <c r="X30" s="515" t="n"/>
+      <c r="Y30" s="513" t="n"/>
+      <c r="Z30" s="514" t="n"/>
+      <c r="AA30" s="514" t="n"/>
+      <c r="AB30" s="514" t="n"/>
+      <c r="AC30" s="515" t="n"/>
+      <c r="AD30" s="516" t="n"/>
+      <c r="AE30" s="514" t="n"/>
+      <c r="AF30" s="514" t="n"/>
+      <c r="AG30" s="514" t="n"/>
+      <c r="AH30" s="515" t="n"/>
+      <c r="AI30" s="517" t="n"/>
+      <c r="AJ30" s="517" t="n"/>
+      <c r="AK30" s="518" t="n"/>
+      <c r="AL30" s="519" t="n"/>
+    </row>
+    <row r="31" hidden="1" ht="21" customHeight="1">
+      <c r="B31" s="520" t="n"/>
+      <c r="C31" s="521" t="n"/>
+      <c r="D31" s="522" t="n"/>
+      <c r="E31" s="523" t="n"/>
+      <c r="F31" s="523" t="n"/>
+      <c r="G31" s="523" t="n"/>
+      <c r="H31" s="523" t="n"/>
+      <c r="I31" s="7" t="n"/>
+      <c r="J31" s="524" t="n"/>
+      <c r="K31" s="525" t="n"/>
+      <c r="L31" s="525" t="n"/>
+      <c r="M31" s="525" t="n"/>
+      <c r="N31" s="526" t="n"/>
+      <c r="O31" s="524" t="n"/>
+      <c r="P31" s="525" t="n"/>
+      <c r="Q31" s="525" t="n"/>
+      <c r="R31" s="525" t="n"/>
+      <c r="S31" s="526" t="n"/>
+      <c r="T31" s="524" t="n"/>
+      <c r="U31" s="525" t="n"/>
+      <c r="V31" s="525" t="n"/>
+      <c r="W31" s="525" t="n"/>
+      <c r="X31" s="526" t="n"/>
+      <c r="Y31" s="524" t="n"/>
+      <c r="Z31" s="525" t="n"/>
+      <c r="AA31" s="525" t="n"/>
+      <c r="AB31" s="525" t="n"/>
+      <c r="AC31" s="526" t="n"/>
+      <c r="AD31" s="524" t="n"/>
+      <c r="AE31" s="525" t="n"/>
+      <c r="AF31" s="525" t="n"/>
+      <c r="AG31" s="525" t="n"/>
+      <c r="AH31" s="526" t="n"/>
+      <c r="AI31" s="527" t="n"/>
+      <c r="AJ31" s="528" t="n"/>
+      <c r="AK31" s="7" t="n"/>
+      <c r="AL31" s="529" t="n"/>
+    </row>
+    <row r="32" hidden="1">
+      <c r="B32" s="530" t="n"/>
+      <c r="C32" s="531" t="n"/>
+      <c r="D32" s="532" t="n"/>
+      <c r="E32" s="533" t="n"/>
+      <c r="F32" s="533" t="n"/>
+      <c r="G32" s="533" t="n"/>
+      <c r="H32" s="533" t="n"/>
+      <c r="I32" s="534" t="n"/>
+      <c r="J32" s="535" t="n"/>
+      <c r="K32" s="536" t="n"/>
+      <c r="L32" s="536" t="n"/>
+      <c r="M32" s="536" t="n"/>
+      <c r="N32" s="537" t="n"/>
+      <c r="O32" s="535" t="n"/>
+      <c r="P32" s="536" t="n"/>
+      <c r="Q32" s="536" t="n"/>
+      <c r="R32" s="536" t="n"/>
+      <c r="S32" s="537" t="n"/>
+      <c r="T32" s="535" t="n"/>
+      <c r="U32" s="536" t="n"/>
+      <c r="V32" s="536" t="n"/>
+      <c r="W32" s="536" t="n"/>
+      <c r="X32" s="537" t="n"/>
+      <c r="Y32" s="535" t="n"/>
+      <c r="Z32" s="536" t="n"/>
+      <c r="AA32" s="536" t="n"/>
+      <c r="AB32" s="536" t="n"/>
+      <c r="AC32" s="537" t="n"/>
+      <c r="AD32" s="538" t="n"/>
+      <c r="AE32" s="536" t="n"/>
+      <c r="AF32" s="536" t="n"/>
+      <c r="AG32" s="536" t="n"/>
+      <c r="AH32" s="537" t="n"/>
+      <c r="AI32" s="539" t="n"/>
+      <c r="AJ32" s="540" t="n"/>
+      <c r="AK32" s="541" t="n"/>
+      <c r="AL32" s="542" t="n"/>
+    </row>
+    <row r="33" hidden="1">
+      <c r="B33" s="530" t="n"/>
+      <c r="C33" s="543" t="n"/>
+      <c r="D33" s="544" t="n"/>
+      <c r="E33" s="545" t="n"/>
+      <c r="F33" s="545" t="n"/>
+      <c r="G33" s="545" t="n"/>
+      <c r="H33" s="545" t="n"/>
+      <c r="I33" s="534" t="n"/>
+      <c r="J33" s="546" t="n"/>
+      <c r="K33" s="547" t="n"/>
+      <c r="L33" s="547" t="n"/>
+      <c r="M33" s="547" t="n"/>
+      <c r="N33" s="537" t="n"/>
+      <c r="O33" s="546" t="n"/>
+      <c r="P33" s="547" t="n"/>
+      <c r="Q33" s="547" t="n"/>
+      <c r="R33" s="547" t="n"/>
+      <c r="S33" s="548" t="n"/>
+      <c r="T33" s="546" t="n"/>
+      <c r="U33" s="547" t="n"/>
+      <c r="V33" s="547" t="n"/>
+      <c r="W33" s="547" t="n"/>
+      <c r="X33" s="548" t="n"/>
+      <c r="Y33" s="546" t="n"/>
+      <c r="Z33" s="547" t="n"/>
+      <c r="AA33" s="547" t="n"/>
+      <c r="AB33" s="547" t="n"/>
+      <c r="AC33" s="548" t="n"/>
+      <c r="AD33" s="538" t="n"/>
+      <c r="AE33" s="547" t="n"/>
+      <c r="AF33" s="547" t="n"/>
+      <c r="AG33" s="547" t="n"/>
+      <c r="AH33" s="548" t="n"/>
+      <c r="AI33" s="549" t="n"/>
+      <c r="AJ33" s="540" t="n"/>
+      <c r="AK33" s="541" t="n"/>
+      <c r="AL33" s="542" t="n"/>
+    </row>
+    <row r="34" hidden="1" ht="19.5" customHeight="1" thickBot="1">
+      <c r="B34" s="550" t="n"/>
+      <c r="C34" s="551" t="n"/>
+      <c r="D34" s="552" t="n"/>
+      <c r="E34" s="553" t="n"/>
+      <c r="F34" s="553" t="n"/>
+      <c r="G34" s="553" t="n"/>
+      <c r="H34" s="553" t="n"/>
+      <c r="I34" s="554" t="n"/>
+      <c r="J34" s="555" t="n"/>
+      <c r="K34" s="556" t="n"/>
+      <c r="L34" s="556" t="n"/>
+      <c r="M34" s="556" t="n"/>
+      <c r="N34" s="557" t="n"/>
+      <c r="O34" s="555" t="n"/>
+      <c r="P34" s="556" t="n"/>
+      <c r="Q34" s="556" t="n"/>
+      <c r="R34" s="556" t="n"/>
+      <c r="S34" s="557" t="n"/>
+      <c r="T34" s="555" t="n"/>
+      <c r="U34" s="556" t="n"/>
+      <c r="V34" s="556" t="n"/>
+      <c r="W34" s="556" t="n"/>
+      <c r="X34" s="557" t="n"/>
+      <c r="Y34" s="555" t="n"/>
+      <c r="Z34" s="556" t="n"/>
+      <c r="AA34" s="556" t="n"/>
+      <c r="AB34" s="556" t="n"/>
+      <c r="AC34" s="557" t="n"/>
+      <c r="AD34" s="555" t="n"/>
+      <c r="AE34" s="556" t="n"/>
+      <c r="AF34" s="556" t="n"/>
+      <c r="AG34" s="556" t="n"/>
+      <c r="AH34" s="557" t="n"/>
+      <c r="AI34" s="558" t="n"/>
+      <c r="AJ34" s="559" t="n"/>
+      <c r="AK34" s="560" t="n"/>
+      <c r="AL34" s="561" t="n"/>
+    </row>
+    <row r="35" hidden="1" customFormat="1" s="119">
+      <c r="D35" s="1" t="n"/>
+      <c r="E35" s="1" t="n"/>
+      <c r="F35" s="1" t="n"/>
+      <c r="G35" s="1" t="n"/>
+      <c r="H35" s="1" t="n"/>
+      <c r="I35" s="1" t="n"/>
+      <c r="J35" s="1" t="n"/>
+      <c r="K35" s="1" t="n"/>
+      <c r="L35" s="1" t="n"/>
+      <c r="M35" s="1" t="n"/>
+      <c r="N35" s="1" t="n"/>
+      <c r="O35" s="1" t="n"/>
+      <c r="P35" s="1" t="n"/>
+      <c r="Q35" s="1" t="n"/>
+      <c r="R35" s="1" t="n"/>
+      <c r="S35" s="1" t="n"/>
+      <c r="T35" s="1" t="n"/>
+      <c r="U35" s="1" t="n"/>
+      <c r="V35" s="1" t="n"/>
+      <c r="W35" s="1" t="n"/>
+      <c r="X35" s="1" t="n"/>
+      <c r="Y35" s="1" t="n"/>
+      <c r="Z35" s="1" t="n"/>
+      <c r="AA35" s="1" t="n"/>
+      <c r="AB35" s="1" t="n"/>
+      <c r="AC35" s="1" t="n"/>
+      <c r="AD35" s="1" t="n"/>
+      <c r="AE35" s="1" t="n"/>
+      <c r="AF35" s="1" t="n"/>
+      <c r="AG35" s="1" t="n"/>
+      <c r="AH35" s="1" t="n"/>
+      <c r="AI35" s="1" t="n"/>
+      <c r="AJ35" s="1" t="n"/>
+      <c r="AK35" s="388" t="n"/>
+      <c r="AL35" s="120" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="39">
+    <mergeCell ref="AD12:AH12"/>
+    <mergeCell ref="T15:X15"/>
+    <mergeCell ref="D3:AJ6"/>
+    <mergeCell ref="O15:S15"/>
+    <mergeCell ref="J14:N14"/>
+    <mergeCell ref="T14:X14"/>
+    <mergeCell ref="AK11:AK17"/>
+    <mergeCell ref="I14:I16"/>
+    <mergeCell ref="Y15:AC15"/>
+    <mergeCell ref="AD14:AH14"/>
+    <mergeCell ref="J13:N13"/>
+    <mergeCell ref="AD13:AH13"/>
+    <mergeCell ref="J15:N15"/>
+    <mergeCell ref="Y11:AC11"/>
+    <mergeCell ref="Y14:AC14"/>
+    <mergeCell ref="AD15:AH15"/>
+    <mergeCell ref="B2:AJ2"/>
+    <mergeCell ref="O16:S16"/>
+    <mergeCell ref="T12:X12"/>
+    <mergeCell ref="J11:N11"/>
+    <mergeCell ref="Y16:AC16"/>
+    <mergeCell ref="J16:N16"/>
+    <mergeCell ref="T11:X11"/>
+    <mergeCell ref="AD11:AH11"/>
+    <mergeCell ref="AI11:AJ17"/>
+    <mergeCell ref="Y13:AC13"/>
+    <mergeCell ref="T13:X13"/>
+    <mergeCell ref="O12:S12"/>
+    <mergeCell ref="Y12:AC12"/>
+    <mergeCell ref="T16:X16"/>
+    <mergeCell ref="B11:H17"/>
+    <mergeCell ref="J12:N12"/>
+    <mergeCell ref="O11:S11"/>
+    <mergeCell ref="AD16:AH16"/>
+    <mergeCell ref="D9:AL9"/>
+    <mergeCell ref="AL11:AL17"/>
+    <mergeCell ref="O14:S14"/>
+    <mergeCell ref="D8:AL8"/>
+    <mergeCell ref="O13:S13"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1" verticalCentered="1"/>
+  <pageMargins left="0.2362204724409449" right="0.1181102362204725" top="0.1574803149606299" bottom="0.1574803149606299" header="0.1968503937007874" footer="0.1574803149606299"/>
+  <pageSetup orientation="landscape" paperSize="9" scale="56" horizontalDpi="4294967293" verticalDpi="4294967293"/>
+  <headerFooter>
+    <oddHeader>&amp;CChampionnat du Tir de precission - REPECHAGE</oddHeader>
+    <oddFooter/>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FFFFC000"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="B1:AI19"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="29" defaultRowHeight="28.5"/>
+  <cols>
+    <col width="8.5703125" customWidth="1" style="564" min="1" max="1"/>
+    <col width="3" customWidth="1" style="564" min="2" max="2"/>
+    <col width="7.7109375" customWidth="1" style="570" min="3" max="3"/>
+    <col width="33.7109375" customWidth="1" style="566" min="4" max="4"/>
+    <col width="28.7109375" customWidth="1" style="578" min="5" max="5"/>
+    <col width="6.28515625" customWidth="1" style="582" min="6" max="7"/>
+    <col width="7" bestFit="1" customWidth="1" style="582" min="8" max="10"/>
+    <col width="6" bestFit="1" customWidth="1" style="582" min="11" max="11"/>
+    <col width="7" bestFit="1" customWidth="1" style="582" min="12" max="12"/>
+    <col width="12" customWidth="1" style="582" min="13" max="13"/>
+    <col width="20.85546875" customWidth="1" style="578" min="14" max="14"/>
+    <col width="6.5703125" customWidth="1" style="578" min="15" max="19"/>
+    <col width="8.7109375" customWidth="1" style="569" min="20" max="20"/>
+    <col width="20.5703125" customWidth="1" style="569" min="21" max="21"/>
+    <col width="6.7109375" customWidth="1" style="569" min="22" max="26"/>
+    <col width="13" bestFit="1" customWidth="1" style="564" min="27" max="27"/>
+    <col width="2" customWidth="1" style="564" min="28" max="28"/>
+    <col width="3.7109375" customWidth="1" style="564" min="29" max="29"/>
+    <col width="29" customWidth="1" style="564" min="30" max="16384"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="84.75" customHeight="1">
+      <c r="B1" s="562" t="n"/>
+      <c r="C1" s="563" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FINAL -Precision shooting  / Tir de précision </t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16.15" customHeight="1" thickBot="1">
+      <c r="C2" s="565" t="n"/>
+      <c r="E2" s="567" t="n"/>
+      <c r="F2" s="568" t="n"/>
+      <c r="G2" s="568" t="n"/>
+      <c r="H2" s="568" t="n"/>
+      <c r="I2" s="568" t="n"/>
+      <c r="J2" s="568" t="n"/>
+      <c r="K2" s="568" t="n"/>
+      <c r="L2" s="568" t="n"/>
+      <c r="M2" s="568" t="n"/>
+      <c r="N2" s="567" t="n"/>
+      <c r="O2" s="567" t="n"/>
+      <c r="P2" s="567" t="n"/>
+      <c r="Q2" s="567" t="n"/>
+      <c r="R2" s="567" t="n"/>
+      <c r="S2" s="567" t="n"/>
+    </row>
+    <row r="3" ht="35.25" customHeight="1" thickBot="1">
+      <c r="D3" s="571" t="n"/>
+      <c r="E3" s="572" t="inlineStr">
+        <is>
+          <t>1/4 Final</t>
+        </is>
+      </c>
+      <c r="F3" s="573" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="G3" s="574" t="inlineStr">
+        <is>
+          <t>REP</t>
+        </is>
+      </c>
+      <c r="H3" s="576" t="n"/>
+      <c r="I3" s="723" t="n"/>
+      <c r="J3" s="723" t="n"/>
+      <c r="K3" s="723" t="n"/>
+      <c r="L3" s="724" t="n"/>
+      <c r="M3" s="577" t="inlineStr">
+        <is>
+          <t>SCORE</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="6.75" customHeight="1" thickBot="1">
+      <c r="F4" s="579" t="n"/>
+      <c r="G4" s="580" t="n"/>
+      <c r="H4" s="581" t="n"/>
+      <c r="I4" s="581" t="n"/>
+      <c r="J4" s="581" t="n"/>
+      <c r="K4" s="581" t="n"/>
+      <c r="L4" s="581" t="n"/>
+    </row>
+    <row r="5" ht="65.25" customHeight="1">
+      <c r="C5" s="583" t="n"/>
+      <c r="D5" s="584" t="n"/>
+      <c r="E5" s="585" t="n"/>
+      <c r="F5" s="586" t="n"/>
+      <c r="G5" s="587" t="n"/>
+      <c r="H5" s="588" t="n"/>
+      <c r="I5" s="589" t="n"/>
+      <c r="J5" s="589" t="n"/>
+      <c r="K5" s="589" t="n"/>
+      <c r="L5" s="590" t="n"/>
+      <c r="M5" s="591" t="n"/>
+      <c r="T5" s="564" t="n"/>
+      <c r="U5" s="564" t="n"/>
+      <c r="V5" s="564" t="n"/>
+      <c r="W5" s="564" t="n"/>
+      <c r="X5" s="564" t="n"/>
+      <c r="Y5" s="564" t="n"/>
+      <c r="Z5" s="564" t="n"/>
+    </row>
+    <row r="6" ht="65.25" customHeight="1" thickBot="1">
+      <c r="C6" s="592" t="n"/>
+      <c r="D6" s="593" t="n"/>
+      <c r="E6" s="594" t="n"/>
+      <c r="F6" s="595" t="n"/>
+      <c r="G6" s="596" t="n"/>
+      <c r="H6" s="597" t="n"/>
+      <c r="I6" s="598" t="n"/>
+      <c r="J6" s="598" t="n"/>
+      <c r="K6" s="598" t="n"/>
+      <c r="L6" s="599" t="n"/>
+      <c r="M6" s="600" t="n"/>
+      <c r="N6" s="601" t="inlineStr">
+        <is>
+          <t>1/2 Final</t>
+        </is>
+      </c>
+      <c r="O6" s="602" t="n"/>
+      <c r="P6" s="602" t="n"/>
+      <c r="Q6" s="602" t="n"/>
+      <c r="R6" s="602" t="n"/>
+      <c r="S6" s="602" t="n"/>
+      <c r="T6" s="602" t="n"/>
+      <c r="U6" s="564" t="n"/>
+      <c r="V6" s="564" t="n"/>
+      <c r="W6" s="564" t="n"/>
+      <c r="X6" s="564" t="n"/>
+      <c r="Y6" s="564" t="n"/>
+      <c r="Z6" s="564" t="n"/>
+    </row>
+    <row r="7" ht="65.25" customHeight="1" thickBot="1">
+      <c r="C7" s="603" t="n"/>
+      <c r="D7" s="604" t="n"/>
+      <c r="E7" s="605" t="n"/>
+      <c r="F7" s="606" t="n"/>
+      <c r="G7" s="606" t="n"/>
+      <c r="H7" s="607" t="n"/>
+      <c r="I7" s="607" t="n"/>
+      <c r="J7" s="607" t="n"/>
+      <c r="K7" s="607" t="n"/>
+      <c r="L7" s="607" t="n"/>
+      <c r="M7" s="608" t="n"/>
+      <c r="N7" s="609" t="n"/>
+      <c r="O7" s="588" t="n"/>
+      <c r="P7" s="589" t="n"/>
+      <c r="Q7" s="589" t="n"/>
+      <c r="R7" s="589" t="n"/>
+      <c r="S7" s="590" t="n"/>
+      <c r="T7" s="610" t="n"/>
+      <c r="U7" s="564" t="n"/>
+      <c r="V7" s="564" t="n"/>
+      <c r="W7" s="564" t="n"/>
+      <c r="X7" s="564" t="n"/>
+      <c r="Y7" s="564" t="n"/>
+      <c r="Z7" s="564" t="n"/>
+    </row>
+    <row r="8" ht="65.25" customHeight="1" thickBot="1" thickTop="1">
+      <c r="C8" s="603" t="n"/>
+      <c r="D8" s="611" t="n"/>
+      <c r="E8" s="612" t="n"/>
+      <c r="F8" s="606" t="n"/>
+      <c r="G8" s="606" t="n"/>
+      <c r="H8" s="607" t="n"/>
+      <c r="I8" s="607" t="n"/>
+      <c r="J8" s="607" t="n"/>
+      <c r="K8" s="607" t="n"/>
+      <c r="L8" s="607" t="n"/>
+      <c r="M8" s="613" t="n"/>
+      <c r="N8" s="614" t="n"/>
+      <c r="O8" s="597" t="n"/>
+      <c r="P8" s="598" t="n"/>
+      <c r="Q8" s="598" t="n"/>
+      <c r="R8" s="598" t="n"/>
+      <c r="S8" s="599" t="n"/>
+      <c r="T8" s="615" t="n"/>
+      <c r="U8" s="616" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="V8" s="725" t="n"/>
+      <c r="W8" s="725" t="n"/>
+      <c r="X8" s="725" t="n"/>
+      <c r="Y8" s="725" t="n"/>
+      <c r="Z8" s="725" t="n"/>
+      <c r="AA8" s="725" t="n"/>
+    </row>
+    <row r="9" ht="65.25" customHeight="1">
+      <c r="C9" s="583" t="n"/>
+      <c r="D9" s="584" t="n"/>
+      <c r="E9" s="585" t="n"/>
+      <c r="F9" s="586" t="n"/>
+      <c r="G9" s="587" t="n"/>
+      <c r="H9" s="588" t="n"/>
+      <c r="I9" s="589" t="n"/>
+      <c r="J9" s="589" t="n"/>
+      <c r="K9" s="589" t="n"/>
+      <c r="L9" s="590" t="n"/>
+      <c r="M9" s="591" t="n"/>
+      <c r="N9" s="618" t="n"/>
+      <c r="T9" s="619" t="n"/>
+      <c r="U9" s="620" t="n"/>
+      <c r="V9" s="621" t="n"/>
+      <c r="W9" s="622" t="n"/>
+      <c r="X9" s="622" t="n"/>
+      <c r="Y9" s="622" t="n"/>
+      <c r="Z9" s="623" t="n"/>
+      <c r="AA9" s="624" t="n"/>
+    </row>
+    <row r="10" ht="65.25" customHeight="1" thickBot="1">
+      <c r="C10" s="592" t="n"/>
+      <c r="D10" s="593" t="n"/>
+      <c r="E10" s="625" t="n"/>
+      <c r="F10" s="595" t="n"/>
+      <c r="G10" s="596" t="n"/>
+      <c r="H10" s="597" t="n"/>
+      <c r="I10" s="598" t="n"/>
+      <c r="J10" s="598" t="n"/>
+      <c r="K10" s="598" t="n"/>
+      <c r="L10" s="599" t="n"/>
+      <c r="M10" s="600" t="n"/>
+      <c r="N10" s="618" t="n"/>
+      <c r="T10" s="619" t="n"/>
+      <c r="U10" s="709" t="n"/>
+      <c r="V10" s="726" t="n"/>
+      <c r="W10" s="727" t="n"/>
+      <c r="X10" s="727" t="n"/>
+      <c r="Y10" s="727" t="n"/>
+      <c r="Z10" s="728" t="n"/>
+      <c r="AA10" s="713" t="n"/>
+      <c r="AI10" s="631" t="n"/>
+    </row>
+    <row r="11" ht="65.25" customHeight="1" thickBot="1">
+      <c r="C11" s="603" t="n"/>
+      <c r="D11" s="604" t="n"/>
+      <c r="E11" s="605" t="n"/>
+      <c r="F11" s="606" t="n"/>
+      <c r="G11" s="606" t="n"/>
+      <c r="H11" s="607" t="n"/>
+      <c r="I11" s="607" t="n"/>
+      <c r="J11" s="607" t="n"/>
+      <c r="K11" s="607" t="n"/>
+      <c r="L11" s="607" t="n"/>
+      <c r="M11" s="608" t="n"/>
+      <c r="N11" s="632" t="n"/>
+      <c r="O11" s="562" t="n"/>
+      <c r="P11" s="562" t="n"/>
+      <c r="Q11" s="562" t="n"/>
+      <c r="R11" s="562" t="n"/>
+      <c r="T11" s="633" t="n"/>
+      <c r="U11" s="729" t="n"/>
+      <c r="V11" s="730" t="n"/>
+      <c r="W11" s="730" t="n"/>
+      <c r="X11" s="730" t="n"/>
+      <c r="Y11" s="730" t="n"/>
+      <c r="Z11" s="730" t="n"/>
+      <c r="AA11" s="731" t="n"/>
+    </row>
+    <row r="12" ht="65.25" customHeight="1" thickBot="1">
+      <c r="C12" s="603" t="n"/>
+      <c r="D12" s="611" t="n"/>
+      <c r="E12" s="637" t="n"/>
+      <c r="F12" s="638" t="n"/>
+      <c r="G12" s="638" t="n"/>
+      <c r="H12" s="639" t="n"/>
+      <c r="I12" s="639" t="n"/>
+      <c r="J12" s="639" t="n"/>
+      <c r="K12" s="639" t="n"/>
+      <c r="L12" s="639" t="n"/>
+      <c r="M12" s="640" t="n"/>
+      <c r="N12" s="618" t="n"/>
+      <c r="O12" s="641" t="n"/>
+      <c r="P12" s="641" t="n"/>
+      <c r="Q12" s="641" t="n"/>
+      <c r="R12" s="641" t="n"/>
+      <c r="S12" s="641" t="n"/>
+      <c r="T12" s="642" t="n"/>
+      <c r="AA12" s="643" t="n"/>
+    </row>
+    <row r="13" ht="65.25" customHeight="1">
+      <c r="C13" s="583" t="n"/>
+      <c r="D13" s="584" t="n"/>
+      <c r="E13" s="585" t="n"/>
+      <c r="F13" s="586" t="n"/>
+      <c r="G13" s="587" t="n"/>
+      <c r="H13" s="588" t="n"/>
+      <c r="I13" s="589" t="n"/>
+      <c r="J13" s="589" t="n"/>
+      <c r="K13" s="589" t="n"/>
+      <c r="L13" s="590" t="n"/>
+      <c r="M13" s="591" t="n"/>
+      <c r="N13" s="644" t="n"/>
+      <c r="O13" s="645" t="n"/>
+      <c r="P13" s="645" t="n"/>
+      <c r="Q13" s="645" t="n"/>
+      <c r="R13" s="645" t="n"/>
+      <c r="S13" s="645" t="n"/>
+      <c r="T13" s="619" t="n"/>
+      <c r="U13" s="732" t="n"/>
+      <c r="V13" s="621" t="n"/>
+      <c r="W13" s="622" t="n"/>
+      <c r="X13" s="622" t="n"/>
+      <c r="Y13" s="622" t="n"/>
+      <c r="Z13" s="623" t="n"/>
+      <c r="AA13" s="624" t="n"/>
+    </row>
+    <row r="14" ht="65.25" customHeight="1" thickBot="1">
+      <c r="C14" s="592" t="n"/>
+      <c r="D14" s="647" t="n"/>
+      <c r="E14" s="594" t="n"/>
+      <c r="F14" s="595" t="n"/>
+      <c r="G14" s="596" t="n"/>
+      <c r="H14" s="597" t="n"/>
+      <c r="I14" s="598" t="n"/>
+      <c r="J14" s="598" t="n"/>
+      <c r="K14" s="598" t="n"/>
+      <c r="L14" s="599" t="n"/>
+      <c r="M14" s="600" t="n"/>
+      <c r="N14" s="648" t="n"/>
+      <c r="O14" s="649" t="n"/>
+      <c r="P14" s="649" t="n"/>
+      <c r="Q14" s="649" t="n"/>
+      <c r="R14" s="649" t="n"/>
+      <c r="S14" s="649" t="n"/>
+      <c r="T14" s="619" t="n"/>
+      <c r="U14" s="733" t="n"/>
+      <c r="V14" s="726" t="n"/>
+      <c r="W14" s="727" t="n"/>
+      <c r="X14" s="727" t="n"/>
+      <c r="Y14" s="727" t="n"/>
+      <c r="Z14" s="728" t="n"/>
+      <c r="AA14" s="713" t="n"/>
+      <c r="AI14" s="631" t="n"/>
+    </row>
+    <row r="15" ht="65.25" customHeight="1" thickBot="1">
+      <c r="C15" s="603" t="n"/>
+      <c r="D15" s="604" t="n"/>
+      <c r="E15" s="654" t="n"/>
+      <c r="F15" s="655" t="n"/>
+      <c r="G15" s="655" t="n"/>
+      <c r="H15" s="656" t="n"/>
+      <c r="I15" s="656" t="n"/>
+      <c r="J15" s="656" t="n"/>
+      <c r="K15" s="656" t="n"/>
+      <c r="L15" s="656" t="n"/>
+      <c r="M15" s="657" t="n"/>
+      <c r="N15" s="609" t="n"/>
+      <c r="O15" s="588" t="n"/>
+      <c r="P15" s="589" t="n"/>
+      <c r="Q15" s="589" t="n"/>
+      <c r="R15" s="589" t="n"/>
+      <c r="S15" s="590" t="n"/>
+      <c r="T15" s="610" t="n"/>
+      <c r="U15" s="734" t="n"/>
+      <c r="V15" s="730" t="n"/>
+      <c r="W15" s="730" t="n"/>
+      <c r="X15" s="730" t="n"/>
+      <c r="Y15" s="730" t="n"/>
+      <c r="Z15" s="730" t="n"/>
+      <c r="AA15" s="731" t="n"/>
+    </row>
+    <row r="16" ht="65.25" customHeight="1" thickBot="1" thickTop="1">
+      <c r="C16" s="603" t="n"/>
+      <c r="D16" s="611" t="n"/>
+      <c r="E16" s="661" t="n"/>
+      <c r="F16" s="606" t="n"/>
+      <c r="G16" s="606" t="n"/>
+      <c r="H16" s="607" t="n"/>
+      <c r="I16" s="607" t="n"/>
+      <c r="J16" s="607" t="n"/>
+      <c r="K16" s="607" t="n"/>
+      <c r="L16" s="607" t="n"/>
+      <c r="M16" s="613" t="n"/>
+      <c r="N16" s="614" t="n"/>
+      <c r="O16" s="597" t="n"/>
+      <c r="P16" s="598" t="n"/>
+      <c r="Q16" s="598" t="n"/>
+      <c r="R16" s="598" t="n"/>
+      <c r="S16" s="599" t="n"/>
+      <c r="T16" s="615" t="n"/>
+    </row>
+    <row r="17" ht="65.25" customHeight="1">
+      <c r="C17" s="583" t="n"/>
+      <c r="D17" s="584" t="n"/>
+      <c r="E17" s="585" t="n"/>
+      <c r="F17" s="586" t="n"/>
+      <c r="G17" s="587" t="n"/>
+      <c r="H17" s="588" t="n"/>
+      <c r="I17" s="589" t="n"/>
+      <c r="J17" s="589" t="n"/>
+      <c r="K17" s="589" t="n"/>
+      <c r="L17" s="590" t="n"/>
+      <c r="M17" s="591" t="n"/>
+      <c r="N17" s="662" t="n">
+        <v>39</v>
+      </c>
+      <c r="T17" s="564" t="n"/>
+      <c r="U17" s="564" t="n"/>
+      <c r="V17" s="564" t="n"/>
+      <c r="W17" s="564" t="n"/>
+      <c r="X17" s="564" t="n"/>
+      <c r="Y17" s="564" t="n"/>
+      <c r="Z17" s="564" t="n"/>
+    </row>
+    <row r="18" ht="65.25" customHeight="1" thickBot="1">
+      <c r="C18" s="592" t="n"/>
+      <c r="D18" s="593" t="n"/>
+      <c r="E18" s="625" t="n"/>
+      <c r="F18" s="595" t="n"/>
+      <c r="G18" s="596" t="n"/>
+      <c r="H18" s="597" t="n"/>
+      <c r="I18" s="598" t="n"/>
+      <c r="J18" s="598" t="n"/>
+      <c r="K18" s="598" t="n"/>
+      <c r="L18" s="599" t="n"/>
+      <c r="M18" s="600" t="n"/>
+      <c r="N18" s="662" t="n">
+        <v>36</v>
+      </c>
+      <c r="T18" s="564" t="n"/>
+      <c r="U18" s="564" t="n"/>
+      <c r="V18" s="564" t="n"/>
+      <c r="W18" s="564" t="n"/>
+      <c r="X18" s="564" t="n"/>
+      <c r="Y18" s="564" t="n"/>
+      <c r="Z18" s="564" t="n"/>
+    </row>
+    <row r="19" ht="14.25" customHeight="1">
+      <c r="E19" s="567" t="n"/>
+      <c r="F19" s="568" t="n"/>
+      <c r="G19" s="568" t="n"/>
+      <c r="H19" s="568" t="n"/>
+      <c r="I19" s="568" t="n"/>
+      <c r="J19" s="568" t="n"/>
+      <c r="K19" s="568" t="n"/>
+      <c r="L19" s="568" t="n"/>
+      <c r="M19" s="568" t="n"/>
+      <c r="N19" s="567" t="n"/>
+      <c r="O19" s="567" t="n"/>
+      <c r="P19" s="567" t="n"/>
+      <c r="Q19" s="567" t="n"/>
+      <c r="R19" s="567" t="n"/>
+      <c r="S19" s="567" t="n"/>
+    </row>
+    <row r="20" ht="7.9" customHeight="1"/>
+  </sheetData>
+  <mergeCells count="19">
+    <mergeCell ref="Y9:Y10"/>
+    <mergeCell ref="AA9:AA10"/>
+    <mergeCell ref="V13:V14"/>
+    <mergeCell ref="U8:AA8"/>
+    <mergeCell ref="X13:X14"/>
+    <mergeCell ref="V9:V10"/>
+    <mergeCell ref="U13:U14"/>
+    <mergeCell ref="U15:AA15"/>
+    <mergeCell ref="Y13:Y14"/>
+    <mergeCell ref="W9:W10"/>
+    <mergeCell ref="Z13:Z14"/>
+    <mergeCell ref="X9:X10"/>
+    <mergeCell ref="U11:AA11"/>
+    <mergeCell ref="C1:AA1"/>
+    <mergeCell ref="H3:L3"/>
+    <mergeCell ref="Z9:Z10"/>
+    <mergeCell ref="W13:W14"/>
+    <mergeCell ref="U9:U10"/>
+    <mergeCell ref="AA13:AA14"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1" verticalCentered="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" paperSize="9" scale="46"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>